<commit_message>
Intègre le temps de validation des étapes (10% = 1 mois) dans les deux plans
Les comptes directs sont financés immédiatement ; les comptes à étapes ne
rapportent qu'après leur évaluation (objectif/10% en mois, ex. 2 étapes
10%+5% = 1,5 mois). Colonnes capital en évaluation, durée d'évaluation et
date de financement ajoutées. Appliqué à plan-scaling-date.xlsx et
plan-scaling-propfirmmatch.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpnEpdwNF8V8azepdqLgDD
</commit_message>
<xml_diff>
--- a/docs/plan-scaling-propfirmmatch.xlsx
+++ b/docs/plan-scaling-propfirmmatch.xlsx
@@ -60,7 +60,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +80,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -138,13 +143,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -234,7 +241,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Capital financé total</a:t>
+              <a:t>Capital financé (validé)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -248,7 +255,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Plan mensuel'!F1</f>
+              <f>'Plan mensuel'!D1</f>
             </strRef>
           </tx>
           <spPr>
@@ -266,12 +273,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Plan mensuel'!$A$2:$A$5</f>
+              <f>'Plan mensuel'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Plan mensuel'!$F$2:$F$5</f>
+              <f>'Plan mensuel'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -351,7 +358,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Plan mensuel'!I1</f>
+              <f>'Plan mensuel'!H1</f>
             </strRef>
           </tx>
           <spPr>
@@ -369,12 +376,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Plan mensuel'!$A$2:$A$5</f>
+              <f>'Plan mensuel'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Plan mensuel'!$I$2:$I$5</f>
+              <f>'Plan mensuel'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -766,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="116" customWidth="1" min="1" max="1"/>
@@ -775,7 +782,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan de scaling PropFirmMatch — maximum de firmes par mois</t>
+          <t>Plan de scaling PropFirmMatch — avec temps de validation des étapes</t>
         </is>
       </c>
     </row>
@@ -795,76 +802,97 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>VOTRE MÉTHODE</t>
+          <t>VOTRE MÉTHODE + TEMPS DE VALIDATION</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>01 octobre 2026 : compte direct FundedNext 10 000 $. Fin octobre, payout 10 % = 1 000 $, moins 30 % firme = 700 $.</t>
+          <t>01 octobre 2026 : compte direct FundedNext 10 000 $. Fin octobre, payout 10 % = 1 000 $, moins 30 % = 700 $.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Chaque mois, avec tout l'argent disponible, vous achetez le MAXIMUM de firmes possible (pas une seule) : on prend le plus gros capital d'abord, firmes CFD en MetaTrader 5, puis autres CFD, puis Futures, chacune une seule fois. Ce classeur ne contient QUE les firmes listées sur le site PropFirmMatch. Le reste du payout est votre salaire.</t>
+          <t>Chaque mois, tout l'argent disponible achète le maximum de firmes (plus gros capital d'abord ; CFD MetaTrader 5, puis CFD, puis Futures ; chacune une fois).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dans ce scénario (10 % / 30 %), les 85 firmes (≈ 51 M$) sont toutes acquises dès janvier 2027.</t>
+          <t>Comptes DIRECTS / INSTANT : financés immédiatement, ils rapportent dès la fin du mois d'achat.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Comptes À ÉTAPES : il faut d'abord valider l'évaluation, à raison de 10 % par mois. Un objectif de 10 % prend 1 mois, 5 % prend une demi-mois. Un 2 étapes 10 %+5 % met donc 1,5 mois à être financé, et ne rapporte qu'ensuite. La durée exacte est dans l'onglet Détail (colonne Durée d'évaluation) et sa date de financement.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>LES ONGLETS</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Ce classeur ne contient QUE les firmes listées sur le site PropFirmMatch.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Plan mensuel : une ligne par mois (date en lettres), nombre de firmes achetées, capital ajouté, capital total, payout brut, part firme, salaire net, trésorerie.</t>
+          <t>Dans ce scénario (10 % / 30 %), la dernière firme est financée vers le 01 mai 2027.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Détail des achats : une ligne par firme achetée, avec sa date, son cycle, sa plateforme, MT5 ou non, son capital et son prix.</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Paramètres / Graphiques.</t>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>LES ONGLETS</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Plan mensuel : date en lettres, firmes achetées, capital financé (déjà validé), capital en cours d'évaluation, payout brut, part firme, salaire net, trésorerie.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>NOTE</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Détail des achats : chaque firme, sa date d'achat, son type, sa durée d'évaluation et sa date de financement.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>L'ordre et le calendrier des achats sont calculés pour le scénario 10 %/30 %. Les colonnes d'argent sont des formules : changez le payout ou la part firme et salaire, part firme et trésorerie se recalculent. Prix hors codes promo. Borne théorique sans échec d'évaluation ni plafond de retrait.</t>
+          <t>Paramètres / Graphiques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Ordre et calendrier calculés pour 10 %/30 %. Colonnes d'argent en formules. Prix hors codes promo. Borne théorique sans échec d'évaluation ni plafond de retrait.</t>
         </is>
       </c>
     </row>
@@ -934,20 +962,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -968,37 +996,37 @@
       </c>
       <c r="D1" s="8" t="inlineStr">
         <is>
-          <t>Capital ajouté ($)</t>
+          <t>Capital financé (validé) ($)</t>
         </is>
       </c>
       <c r="E1" s="8" t="inlineStr">
         <is>
-          <t>Prix payé ($)</t>
+          <t>Capital en évaluation ($)</t>
         </is>
       </c>
       <c r="F1" s="8" t="inlineStr">
         <is>
-          <t>Capital financé total ($)</t>
+          <t>Payout brut ($)</t>
         </is>
       </c>
       <c r="G1" s="8" t="inlineStr">
         <is>
-          <t>Payout brut ($)</t>
+          <t>Part firme ($)</t>
         </is>
       </c>
       <c r="H1" s="8" t="inlineStr">
         <is>
-          <t>Part firme ($)</t>
+          <t>Salaire net ($)</t>
         </is>
       </c>
       <c r="I1" s="8" t="inlineStr">
         <is>
-          <t>Salaire net ($)</t>
+          <t>Trésorerie ($)</t>
         </is>
       </c>
       <c r="J1" s="8" t="inlineStr">
         <is>
-          <t>Trésorerie ($)</t>
+          <t>Comptes financés</t>
         </is>
       </c>
       <c r="K1" s="8" t="inlineStr">
@@ -1022,29 +1050,29 @@
         <v>1</v>
       </c>
       <c r="D2" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E2" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="11" t="n">
-        <v>10000</v>
-      </c>
-      <c r="G2" s="10">
-        <f>F2*Paramètres!$B$3</f>
+      <c r="F2" s="12">
+        <f>D2*Paramètres!$B$3</f>
         <v/>
       </c>
+      <c r="G2" s="12">
+        <f>F2*Paramètres!$B$4</f>
+        <v/>
+      </c>
       <c r="H2" s="10">
-        <f>G2*Paramètres!$B$4</f>
+        <f>F2-G2</f>
         <v/>
       </c>
-      <c r="I2" s="11">
-        <f>G2-H2</f>
+      <c r="I2" s="12">
+        <f>H2-0</f>
         <v/>
       </c>
-      <c r="J2" s="10">
-        <f>I2-E2</f>
-        <v/>
+      <c r="J2" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="K2" s="9" t="n">
         <v>1</v>
@@ -1065,29 +1093,29 @@
         <v>3</v>
       </c>
       <c r="D3" s="10" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E3" s="11" t="n">
         <v>323000</v>
       </c>
-      <c r="E3" s="10" t="n">
-        <v>686</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <v>333000</v>
-      </c>
-      <c r="G3" s="10">
-        <f>F3*Paramètres!$B$3</f>
+      <c r="F3" s="12">
+        <f>D3*Paramètres!$B$3</f>
         <v/>
       </c>
+      <c r="G3" s="12">
+        <f>F3*Paramètres!$B$4</f>
+        <v/>
+      </c>
       <c r="H3" s="10">
-        <f>G3*Paramètres!$B$4</f>
+        <f>F3-G3</f>
         <v/>
       </c>
-      <c r="I3" s="11">
-        <f>G3-H3</f>
+      <c r="I3" s="12">
+        <f>I2+H3-686</f>
         <v/>
       </c>
-      <c r="J3" s="10">
-        <f>J2+I3-E3</f>
-        <v/>
+      <c r="J3" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="K3" s="9" t="n">
         <v>4</v>
@@ -1101,39 +1129,39 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>PaidPex; Lux Trading Firm; XLTrade; Leveraged; The5ers Crypto</t>
+          <t>The5ers Crypto; Real Trader Fund</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>433000</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>120000</v>
+      </c>
+      <c r="F4" s="12">
+        <f>D4*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>F4*Paramètres!$B$4</f>
+        <v/>
+      </c>
+      <c r="H4" s="10">
+        <f>F4-G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="12">
+        <f>I3+H4-477</f>
+        <v/>
+      </c>
+      <c r="J4" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="10" t="n">
-        <v>13120000</v>
-      </c>
-      <c r="E4" s="10" t="n">
-        <v>23236</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>13453000</v>
-      </c>
-      <c r="G4" s="10">
-        <f>F4*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="H4" s="10">
-        <f>G4*Paramètres!$B$4</f>
-        <v/>
-      </c>
-      <c r="I4" s="11">
-        <f>G4-H4</f>
-        <v/>
-      </c>
-      <c r="J4" s="10">
-        <f>J3+I4-E4</f>
-        <v/>
-      </c>
       <c r="K4" s="9" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1144,38 +1172,202 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Upcomers; Finotive Funding; Funded Trader Markets; IF Crypto; Instant Funding; Sway Funded … (+71)</t>
+          <t>PaidPex; Lux Trading Firm; Finotive Funding; XLTrade; Funded Trader Markets; Sway Funded</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>77</v>
+        <v>6</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>37175000</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>248013</v>
-      </c>
-      <c r="F5" s="11" t="n">
+        <v>1433000</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>14520000</v>
+      </c>
+      <c r="F5" s="12">
+        <f>D5*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>F5*Paramètres!$B$4</f>
+        <v/>
+      </c>
+      <c r="H5" s="10">
+        <f>F5-G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="12">
+        <f>I4+H5-41704</f>
+        <v/>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Upcomers; IF Crypto; Instant Funding; Leveraged; Pro Traders Fund; Mainet Funded … (+15)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>22853000</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>9095000</v>
+      </c>
+      <c r="F6" s="12">
+        <f>D6*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>F6*Paramètres!$B$4</f>
+        <v/>
+      </c>
+      <c r="H6" s="10">
+        <f>F6-G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="12">
+        <f>I5+H6-132467</f>
+        <v/>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>FTMO; TradersFlow; The Trading Pit; Ultimate Traders; BrightFunded; Quant Funded … (+47)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>34288000</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>16340000</v>
+      </c>
+      <c r="F7" s="12">
+        <f>D7*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>F7*Paramètres!$B$4</f>
+        <v/>
+      </c>
+      <c r="H7" s="10">
+        <f>F7-G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="12">
+        <f>I6+H7-96601</f>
+        <v/>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr"/>
+      <c r="C8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>50228000</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>400000</v>
+      </c>
+      <c r="F8" s="12">
+        <f>D8*Paramètres!$B$3</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>F8*Paramètres!$B$4</f>
+        <v/>
+      </c>
+      <c r="H8" s="10">
+        <f>F8-G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="12">
+        <f>I7+H8-0</f>
+        <v/>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>01 mai 2027</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="n">
         <v>50628000</v>
       </c>
-      <c r="G5" s="10">
-        <f>F5*Paramètres!$B$3</f>
+      <c r="E9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="12">
+        <f>D9*Paramètres!$B$3</f>
         <v/>
       </c>
-      <c r="H5" s="10">
-        <f>G5*Paramètres!$B$4</f>
+      <c r="G9" s="12">
+        <f>F9*Paramètres!$B$4</f>
         <v/>
       </c>
-      <c r="I5" s="11">
-        <f>G5-H5</f>
+      <c r="H9" s="10">
+        <f>F9-G9</f>
         <v/>
       </c>
-      <c r="J5" s="10">
-        <f>J4+I5-E5</f>
+      <c r="I9" s="12">
+        <f>I8+H9-0</f>
         <v/>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="J9" s="9" t="n">
+        <v>86</v>
+      </c>
+      <c r="K9" s="9" t="n">
         <v>86</v>
       </c>
     </row>
@@ -1190,50 +1382,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Date d'achat</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Cycle</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Prop firm</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Plateforme</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
-        <is>
-          <t>MetaTrader 5 ?</t>
-        </is>
-      </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>MT5 ?</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>Durée évaluation (mois)</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>Date de financement</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Capital ($)</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Prix ($)</t>
         </is>
@@ -1245,7 +1455,7 @@
           <t>01 novembre 2026</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -1265,10 +1475,23 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>01 décembre 2026</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="J2" s="12" t="n">
         <v>514</v>
       </c>
     </row>
@@ -1278,7 +1501,7 @@
           <t>01 novembre 2026</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -1298,10 +1521,23 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>19 décembre 2026</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="n">
         <v>120000</v>
       </c>
-      <c r="G3" s="10" t="n">
+      <c r="J3" s="12" t="n">
         <v>117</v>
       </c>
     </row>
@@ -1311,7 +1547,7 @@
           <t>01 novembre 2026</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -1331,10 +1567,23 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>16 décembre 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="n">
         <v>3000</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="J4" s="12" t="n">
         <v>55</v>
       </c>
     </row>
@@ -1344,19 +1593,19 @@
           <t>01 décembre 2026</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>PaidPex</t>
+          <t>The5ers Crypto</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>cTrader, TradingView</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1364,11 +1613,24 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>11960</v>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>120000</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="6">
@@ -1377,19 +1639,19 @@
           <t>01 décembre 2026</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Lux Trading Firm</t>
+          <t>Real Trader Fund</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>TradingView</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1397,32 +1659,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>4995</v>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>01 décembre 2026</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>360</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>01 décembre 2026</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
+          <t>01 janvier 2027</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>XLTrade</t>
+          <t>PaidPex</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -1430,32 +1705,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>3168</v>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>11960</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>01 décembre 2026</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
+          <t>01 janvier 2027</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Leveraged</t>
+          <t>Lux Trading Firm</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>TradingView</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1463,32 +1751,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>2996</v>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>4995</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>01 décembre 2026</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
+          <t>01 janvier 2027</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>The5ers Crypto</t>
+          <t>Finotive Funding</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>cTrader, TradingView</t>
+          <t>MetaTrader 5, Match-Trader</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -1496,11 +1797,24 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>120000</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>117</v>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>09 février 2027</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>11200</v>
       </c>
     </row>
     <row r="10">
@@ -1509,19 +1823,19 @@
           <t>01 janvier 2027</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Upcomers</t>
+          <t>XLTrade</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker, DXtr</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1529,11 +1843,24 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
-        <v>4000000</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>30795</v>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>3168</v>
       </c>
     </row>
     <row r="11">
@@ -1542,19 +1869,19 @@
           <t>01 janvier 2027</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Finotive Funding</t>
+          <t>Funded Trader Markets</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader</t>
+          <t>cTrader, Match-Trader, TradeLocker</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1562,11 +1889,24 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F11" s="10" t="n">
-        <v>1400000</v>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>11200</v>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>19 janvier 2027</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>5436</v>
       </c>
     </row>
     <row r="12">
@@ -1575,19 +1915,19 @@
           <t>01 janvier 2027</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Funded Trader Markets</t>
+          <t>Sway Funded</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1595,32 +1935,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>25 février 2027</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="n">
         <v>1000000</v>
       </c>
-      <c r="G12" s="10" t="n">
-        <v>5436</v>
+      <c r="J12" s="12" t="n">
+        <v>4945</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>IF Crypto</t>
+          <t>Upcomers</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>cTrader, Match-Trader, TradeLocker, DXtr</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1628,32 +1981,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F13" s="10" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>7390</v>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>25 février 2027</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>30795</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Instant Funding</t>
+          <t>IF Crypto</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1661,32 +2027,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="n">
         <v>1000000</v>
       </c>
-      <c r="G14" s="10" t="n">
+      <c r="J14" s="12" t="n">
         <v>7390</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Sway Funded</t>
+          <t>Instant Funding</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -1694,32 +2073,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>28 février 2027</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="n">
         <v>1000000</v>
       </c>
-      <c r="G15" s="10" t="n">
-        <v>4945</v>
+      <c r="J15" s="12" t="n">
+        <v>7390</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Pro Traders Fund</t>
+          <t>Leveraged</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1727,27 +2119,40 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>900000</v>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>4197</v>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>2996</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Mainet Funded</t>
+          <t>Pro Traders Fund</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1760,32 +2165,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
-        <v>700000</v>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>2975</v>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>07 mars 2027</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>900000</v>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>4197</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Fintokei</t>
+          <t>Mainet Funded</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradingView</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1793,32 +2211,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>10 mars 2027</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="n">
         <v>700000</v>
       </c>
-      <c r="G18" s="10" t="n">
-        <v>2933</v>
+      <c r="J18" s="12" t="n">
+        <v>2975</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B19" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>ADN Broker</t>
+          <t>Fintokei</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5, cTrader, TradingView</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -1826,32 +2257,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F19" s="10" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>50000</v>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>04 mars 2027</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>700000</v>
+      </c>
+      <c r="J19" s="12" t="n">
+        <v>2933</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Hola Prime</t>
+          <t>ADN Broker</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1859,32 +2303,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n">
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G20" s="10" t="n">
-        <v>1236</v>
+      <c r="J20" s="12" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>E8 Perpetuals</t>
+          <t>Hola Prime</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradeLocker</t>
+          <t>cTrader, Match-Trader, TradeLocker</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -1892,32 +2349,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F21" s="10" t="n">
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>19 février 2027</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G21" s="10" t="n">
-        <v>1300</v>
+      <c r="J21" s="12" t="n">
+        <v>1236</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>E8 Markets</t>
+          <t>E8 Perpetuals</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
+          <t>MetaTrader 5, cTrader, TradeLocker</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -1925,32 +2395,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n">
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G22" s="10" t="n">
+      <c r="J22" s="12" t="n">
         <v>1300</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B23" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Foxx Funded</t>
+          <t>E8 Markets</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -1958,32 +2441,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F23" s="10" t="n">
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>19 février 2027</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G23" s="10" t="n">
-        <v>1990</v>
+      <c r="J23" s="12" t="n">
+        <v>1300</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Quantum Funding</t>
+          <t>Foxx Funded</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1991,32 +2487,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n">
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G24" s="10" t="n">
-        <v>2145</v>
+      <c r="J24" s="12" t="n">
+        <v>1990</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>IC Funded</t>
+          <t>Quantum Funding</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -2024,32 +2533,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F25" s="10" t="n">
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G25" s="10" t="n">
-        <v>2495</v>
+      <c r="J25" s="12" t="n">
+        <v>2145</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Vertex Funding</t>
+          <t>IC Funded</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2057,27 +2579,40 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>16 mars 2027</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G26" s="10" t="n">
-        <v>2525</v>
+      <c r="J26" s="12" t="n">
+        <v>2495</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>FNC Funding</t>
+          <t>Vertex Funding</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -2090,27 +2625,40 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F27" s="10" t="n">
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>16 mars 2027</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G27" s="10" t="n">
-        <v>2625</v>
+      <c r="J27" s="12" t="n">
+        <v>2525</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Blink Funding</t>
+          <t>FNC Funding</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -2123,32 +2671,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G28" s="10" t="n">
-        <v>1800</v>
+      <c r="J28" s="12" t="n">
+        <v>2625</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>SFX Funded</t>
+          <t>Blink Funding</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Match-Trader</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -2156,32 +2717,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F29" s="10" t="n">
-        <v>495000</v>
-      </c>
-      <c r="G29" s="10" t="n">
-        <v>2125</v>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>16 mars 2027</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J29" s="12" t="n">
+        <v>1800</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>XPIPS</t>
+          <t>SFX Funded</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>Match-Trader</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2189,32 +2763,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F30" s="10" t="n">
-        <v>400000</v>
-      </c>
-      <c r="G30" s="10" t="n">
-        <v>1596</v>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>10 mars 2027</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>495000</v>
+      </c>
+      <c r="J30" s="12" t="n">
+        <v>2125</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Blue Guardian</t>
+          <t>XPIPS</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader, TradeLocker,</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
@@ -2222,32 +2809,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F31" s="10" t="n">
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G31" s="10" t="n">
-        <v>1472</v>
+      <c r="J31" s="12" t="n">
+        <v>1596</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B32" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>FTMO</t>
+          <t>Blue Guardian</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradingView</t>
+          <t>MetaTrader 5, Match-Trader, TradeLocker,</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2255,32 +2855,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F32" s="10" t="n">
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G32" s="10" t="n">
-        <v>1996</v>
+      <c r="J32" s="12" t="n">
+        <v>1472</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>TradersFlow</t>
+          <t>Atlas Funded</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>MetaTrader 5, TradeLocker, Rithmic</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
@@ -2288,32 +2901,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F33" s="10" t="n">
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G33" s="10" t="n">
-        <v>2018</v>
+      <c r="J33" s="12" t="n">
+        <v>1182</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>The Trading Pit</t>
+          <t>FTMO</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5, cTrader, TradingView</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
@@ -2321,32 +2947,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F34" s="10" t="n">
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G34" s="10" t="n">
-        <v>2276</v>
+      <c r="J34" s="12" t="n">
+        <v>1996</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B35" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>Ultimate Traders</t>
+          <t>TradersFlow</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
@@ -2354,32 +2993,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F35" s="10" t="n">
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G35" s="10" t="n">
-        <v>1798</v>
+      <c r="J35" s="12" t="n">
+        <v>2018</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>BrightFunded</t>
+          <t>The Trading Pit</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>cTrader, DXtrade</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
@@ -2387,32 +3039,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F36" s="10" t="n">
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G36" s="10" t="n">
-        <v>1894</v>
+      <c r="J36" s="12" t="n">
+        <v>2276</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>Quant Funded</t>
+          <t>Ultimate Traders</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">
@@ -2420,32 +3085,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F37" s="10" t="n">
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G37" s="10" t="n">
-        <v>1996</v>
+      <c r="J37" s="12" t="n">
+        <v>1798</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Audacity Capital</t>
+          <t>BrightFunded</t>
         </is>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, DXtrade</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E38" s="9" t="inlineStr">
@@ -2453,32 +3131,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F38" s="10" t="n">
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>10 avril 2027</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G38" s="10" t="n">
-        <v>2098</v>
+      <c r="J38" s="12" t="n">
+        <v>1894</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>WSFunded</t>
+          <t>Quant Funded</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
@@ -2486,32 +3177,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F39" s="10" t="n">
+      <c r="F39" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G39" s="10" t="n">
-        <v>2236</v>
+      <c r="J39" s="12" t="n">
+        <v>1996</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B40" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Atlas Funded</t>
+          <t>Audacity Capital</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, TradeLocker, Rithmic</t>
+          <t>MetaTrader 5, DXtrade</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
@@ -2519,32 +3223,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F40" s="10" t="n">
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G40" s="10" t="n">
-        <v>1182</v>
+      <c r="J40" s="12" t="n">
+        <v>2098</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>AquaFunded</t>
+          <t>WSFunded</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradeLocker, Rith</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -2552,32 +3269,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F41" s="10" t="n">
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G41" s="10" t="n">
-        <v>1354</v>
+      <c r="J41" s="12" t="n">
+        <v>2236</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Orion Funded</t>
+          <t>AquaFunded</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>MetaTrader 5, cTrader, TradeLocker, Rith</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
@@ -2585,32 +3315,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F42" s="10" t="n">
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>19 avril 2027</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G42" s="10" t="n">
-        <v>1478</v>
+      <c r="J42" s="12" t="n">
+        <v>1354</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B43" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Get Crypto Funded</t>
+          <t>Orion Funded</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -2618,32 +3361,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F43" s="10" t="n">
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>01 mai 2027</t>
+        </is>
+      </c>
+      <c r="I43" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G43" s="10" t="n">
-        <v>1648</v>
+      <c r="J43" s="12" t="n">
+        <v>1478</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Funding Pips</t>
+          <t>Get Crypto Funded</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -2651,32 +3407,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F44" s="10" t="n">
-        <v>300000</v>
-      </c>
-      <c r="G44" s="10" t="n">
-        <v>1332</v>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>25 avril 2027</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>400000</v>
+      </c>
+      <c r="J44" s="12" t="n">
+        <v>1648</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B45" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Clarity Traders</t>
+          <t>Funding Pips</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, TradeLocker</t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -2684,32 +3453,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F45" s="10" t="n">
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I45" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G45" s="10" t="n">
-        <v>1399</v>
+      <c r="J45" s="12" t="n">
+        <v>1332</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B46" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Prop Number One</t>
+          <t>Clarity Traders</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
+          <t>MetaTrader 5, TradeLocker</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
@@ -2717,32 +3499,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F46" s="10" t="n">
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>10 avril 2027</t>
+        </is>
+      </c>
+      <c r="I46" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G46" s="10" t="n">
-        <v>1592</v>
+      <c r="J46" s="12" t="n">
+        <v>1399</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Tradeify 247</t>
+          <t>Prop Number One</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, DXtrade</t>
+          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -2750,32 +3545,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F47" s="10" t="n">
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I47" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G47" s="10" t="n">
-        <v>1740</v>
+      <c r="J47" s="12" t="n">
+        <v>1592</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Myfundedcapital</t>
+          <t>Tradeify 247</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>MetaTrader 5, DXtrade</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -2783,32 +3591,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F48" s="10" t="n">
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I48" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G48" s="10" t="n">
-        <v>1905</v>
+      <c r="J48" s="12" t="n">
+        <v>1740</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B49" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Alpine Funded</t>
+          <t>Myfundedcapital</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -2816,32 +3637,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F49" s="10" t="n">
-        <v>200000</v>
-      </c>
-      <c r="G49" s="10" t="n">
-        <v>839</v>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J49" s="12" t="n">
+        <v>1905</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B50" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>FunderPro</t>
+          <t>Alpine Funded</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>cTrader, TradeLocker</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
@@ -2849,32 +3683,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F50" s="10" t="n">
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G50" s="10" t="n">
-        <v>989</v>
+      <c r="J50" s="12" t="n">
+        <v>839</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Funded Trading Plus</t>
+          <t>FunderPro</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>cTrader, TradeLocker</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -2882,32 +3729,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F51" s="10" t="n">
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>13 avril 2027</t>
+        </is>
+      </c>
+      <c r="I51" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G51" s="10" t="n">
-        <v>999</v>
+      <c r="J51" s="12" t="n">
+        <v>989</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B52" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>CK Capital</t>
+          <t>Funded Trading Plus</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>TradeLocker</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -2915,32 +3775,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F52" s="10" t="n">
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I52" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G52" s="10" t="n">
-        <v>1056</v>
+      <c r="J52" s="12" t="n">
+        <v>999</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>NowTradeFunded</t>
+          <t>CK Capital</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>TradeLocker</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -2948,32 +3821,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F53" s="10" t="n">
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>07 avril 2027</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G53" s="10" t="n">
-        <v>900</v>
+      <c r="J53" s="12" t="n">
+        <v>1056</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Crypto Fund Trader</t>
+          <t>NowTradeFunded</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -2981,32 +3867,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F54" s="10" t="n">
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>22 avril 2027</t>
+        </is>
+      </c>
+      <c r="I54" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G54" s="10" t="n">
-        <v>1250</v>
+      <c r="J54" s="12" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>FX2 Funding</t>
+          <t>Crypto Fund Trader</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>cTrader, DXtrade</t>
+          <t>MetaTrader 5, Match-Trader</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
@@ -3014,27 +3913,40 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F55" s="10" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G55" s="10" t="n">
-        <v>1055</v>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>10 avril 2027</t>
+        </is>
+      </c>
+      <c r="I55" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="J55" s="12" t="n">
+        <v>1250</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B56" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Ment Funding</t>
+          <t>FX2 Funding</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -3047,32 +3959,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F56" s="10" t="n">
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I56" s="12" t="n">
         <v>190000</v>
       </c>
-      <c r="G56" s="10" t="n">
-        <v>7451</v>
+      <c r="J56" s="12" t="n">
+        <v>1055</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Leveraged Crypto</t>
+          <t>Ment Funding</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -3080,32 +4005,45 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F57" s="10" t="n">
-        <v>150000</v>
-      </c>
-      <c r="G57" s="10" t="n">
-        <v>980</v>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I57" s="12" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J57" s="12" t="n">
+        <v>7451</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B58" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Real Trader Fund</t>
+          <t>Leveraged Crypto</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
@@ -3113,20 +4051,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F58" s="10" t="n">
-        <v>100000</v>
-      </c>
-      <c r="G58" s="10" t="n">
-        <v>360</v>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J58" s="12" t="n">
+        <v>980</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3146,20 +4097,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F59" s="10" t="n">
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G59" s="10" t="n">
+      <c r="J59" s="12" t="n">
         <v>699</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B60" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3179,20 +4143,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F60" s="10" t="n">
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G60" s="10" t="n">
+      <c r="J60" s="12" t="n">
         <v>549</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3212,20 +4189,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F61" s="10" t="n">
+      <c r="F61" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G61" s="10" t="n">
+      <c r="J61" s="12" t="n">
         <v>579</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B62" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B62" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3245,20 +4235,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F62" s="10" t="n">
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G62" s="10" t="n">
+      <c r="J62" s="12" t="n">
         <v>589</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B63" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3278,20 +4281,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F63" s="10" t="n">
+      <c r="F63" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H63" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G63" s="10" t="n">
+      <c r="J63" s="12" t="n">
         <v>650</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B64" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3311,20 +4327,33 @@
           <t>Oui</t>
         </is>
       </c>
-      <c r="F64" s="10" t="n">
+      <c r="F64" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="G64" s="10" t="n">
+      <c r="J64" s="12" t="n">
         <v>700</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3344,20 +4373,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F65" s="10" t="n">
+      <c r="F65" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I65" s="12" t="n">
         <v>1000000</v>
       </c>
-      <c r="G65" s="10" t="n">
+      <c r="J65" s="12" t="n">
         <v>349</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B66" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3377,20 +4419,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F66" s="10" t="n">
+      <c r="F66" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H66" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I66" s="12" t="n">
         <v>1000000</v>
       </c>
-      <c r="G66" s="10" t="n">
+      <c r="J66" s="12" t="n">
         <v>6150</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B67" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3410,20 +4465,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F67" s="10" t="n">
+      <c r="F67" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G67" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I67" s="12" t="n">
         <v>800000</v>
       </c>
-      <c r="G67" s="10" t="n">
+      <c r="J67" s="12" t="n">
         <v>3600</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B68" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B68" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3443,20 +4511,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F68" s="10" t="n">
+      <c r="F68" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H68" s="9" t="inlineStr">
+        <is>
+          <t>07 avril 2027</t>
+        </is>
+      </c>
+      <c r="I68" s="12" t="n">
         <v>600000</v>
       </c>
-      <c r="G68" s="10" t="n">
+      <c r="J68" s="12" t="n">
         <v>2360</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3476,20 +4557,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F69" s="10" t="n">
+      <c r="F69" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I69" s="12" t="n">
         <v>500000</v>
       </c>
-      <c r="G69" s="10" t="n">
+      <c r="J69" s="12" t="n">
         <v>2450</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B70" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3509,20 +4603,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F70" s="10" t="n">
+      <c r="F70" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I70" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G70" s="10" t="n">
+      <c r="J70" s="12" t="n">
         <v>2625</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B71" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3542,20 +4649,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F71" s="10" t="n">
+      <c r="F71" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>07 avril 2027</t>
+        </is>
+      </c>
+      <c r="I71" s="12" t="n">
         <v>400000</v>
       </c>
-      <c r="G71" s="10" t="n">
+      <c r="J71" s="12" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B72" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B72" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3575,20 +4695,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F72" s="10" t="n">
+      <c r="F72" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I72" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G72" s="10" t="n">
+      <c r="J72" s="12" t="n">
         <v>1450</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B73" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B73" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3608,20 +4741,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F73" s="10" t="n">
+      <c r="F73" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I73" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="G73" s="10" t="n">
+      <c r="J73" s="12" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3641,20 +4787,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F74" s="10" t="n">
+      <c r="F74" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G74" s="15" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>04 avril 2027</t>
+        </is>
+      </c>
+      <c r="I74" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G74" s="10" t="n">
+      <c r="J74" s="12" t="n">
         <v>700</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B75" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3674,20 +4833,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F75" s="10" t="n">
+      <c r="F75" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G75" s="15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>10 avril 2027</t>
+        </is>
+      </c>
+      <c r="I75" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G75" s="10" t="n">
+      <c r="J75" s="12" t="n">
         <v>899</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B76" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3707,20 +4879,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F76" s="10" t="n">
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G76" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H76" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I76" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G76" s="10" t="n">
+      <c r="J76" s="12" t="n">
         <v>999</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B77" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3740,20 +4925,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F77" s="10" t="n">
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G77" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H77" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G77" s="10" t="n">
+      <c r="J77" s="12" t="n">
         <v>799</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B78" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B78" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3773,20 +4971,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F78" s="10" t="n">
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I78" s="12" t="n">
         <v>100000</v>
       </c>
-      <c r="G78" s="10" t="n">
+      <c r="J78" s="12" t="n">
         <v>650</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B79" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3806,20 +5017,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F79" s="10" t="n">
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="I79" s="12" t="n">
         <v>40000</v>
       </c>
-      <c r="G79" s="10" t="n">
+      <c r="J79" s="12" t="n">
         <v>1980</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B80" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3839,20 +5063,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F80" s="10" t="n">
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I80" s="12" t="n">
         <v>25000</v>
       </c>
-      <c r="G80" s="10" t="n">
+      <c r="J80" s="12" t="n">
         <v>141</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B81" s="14" t="inlineStr">
         <is>
           <t>CFD</t>
         </is>
@@ -3872,20 +5109,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F81" s="10" t="n">
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G81" s="15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>16 avril 2027</t>
+        </is>
+      </c>
+      <c r="I81" s="12" t="n">
         <v>25000</v>
       </c>
-      <c r="G81" s="10" t="n">
+      <c r="J81" s="12" t="n">
         <v>149</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B82" s="14" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
         <is>
           <t>Futures</t>
         </is>
@@ -3905,20 +5155,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F82" s="10" t="n">
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>19 mars 2027</t>
+        </is>
+      </c>
+      <c r="I82" s="12" t="n">
         <v>1650000</v>
       </c>
-      <c r="G82" s="10" t="n">
+      <c r="J82" s="12" t="n">
         <v>2114</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B83" s="14" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
         <is>
           <t>Futures</t>
         </is>
@@ -3938,20 +5201,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F83" s="10" t="n">
+      <c r="F83" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G83" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I83" s="12" t="n">
         <v>900000</v>
       </c>
-      <c r="G83" s="10" t="n">
+      <c r="J83" s="12" t="n">
         <v>672</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B84" s="14" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
         <is>
           <t>Futures</t>
         </is>
@@ -3971,20 +5247,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F84" s="10" t="n">
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G84" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" s="9" t="inlineStr">
+        <is>
+          <t>01 avril 2027</t>
+        </is>
+      </c>
+      <c r="I84" s="12" t="n">
         <v>750000</v>
       </c>
-      <c r="G84" s="10" t="n">
+      <c r="J84" s="12" t="n">
         <v>1445</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B85" s="14" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
         <is>
           <t>Futures</t>
         </is>
@@ -4004,20 +5293,33 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F85" s="10" t="n">
+      <c r="F85" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>19 mars 2027</t>
+        </is>
+      </c>
+      <c r="I85" s="12" t="n">
         <v>750000</v>
       </c>
-      <c r="G85" s="10" t="n">
+      <c r="J85" s="12" t="n">
         <v>1625</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
-        </is>
-      </c>
-      <c r="B86" s="14" t="inlineStr">
+          <t>01 mars 2027</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
         <is>
           <t>Futures</t>
         </is>
@@ -4037,10 +5339,23 @@
           <t>Non</t>
         </is>
       </c>
-      <c r="F86" s="10" t="n">
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G86" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H86" s="9" t="inlineStr">
+        <is>
+          <t>25 avril 2027</t>
+        </is>
+      </c>
+      <c r="I86" s="12" t="n">
         <v>200000</v>
       </c>
-      <c r="G86" s="10" t="n">
+      <c r="J86" s="12" t="n">
         <v>999</v>
       </c>
     </row>
@@ -4059,7 +5374,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Graphiques</t>
         </is>

</xml_diff>

<commit_message>
Ordre d'achat par type de plan : instants, puis 1/2/3/4 étapes
Change l'ordre d'achat des deux plans de scaling (complet et
PropFirmMatch) : on achète désormais d'abord TOUS les comptes
directs/instant, puis tous les 1 étape, puis les 2 étapes, 3 étapes
et 4 étapes+. Le cycle CFD (MetaTrader 5 en premier) reste prioritaire
sur les Futures au sein de chaque type, et le plus gros capital
départage à rang égal.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XpnEpdwNF8V8azepdqLgDD
</commit_message>
<xml_diff>
--- a/docs/plan-scaling-propfirmmatch.xlsx
+++ b/docs/plan-scaling-propfirmmatch.xlsx
@@ -273,12 +273,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Plan mensuel'!$A$2:$A$9</f>
+              <f>'Plan mensuel'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Plan mensuel'!$D$2:$D$9</f>
+              <f>'Plan mensuel'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -376,12 +376,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Plan mensuel'!$A$2:$A$9</f>
+              <f>'Plan mensuel'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Plan mensuel'!$H$2:$H$9</f>
+              <f>'Plan mensuel'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -773,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="116" customWidth="1" min="1" max="1"/>
@@ -816,81 +816,88 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Chaque mois, tout l'argent disponible achète le maximum de firmes (plus gros capital d'abord ; CFD MetaTrader 5, puis CFD, puis Futures ; chacune une fois).</t>
+          <t>Chaque mois, tout l'argent disponible achète le maximum de firmes (chacune une fois).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Comptes DIRECTS / INSTANT : financés immédiatement, ils rapportent dès la fin du mois d'achat.</t>
+          <t>ORDRE D'ACHAT : d'abord tous les comptes DIRECTS / INSTANT, puis tous les 1 étape, puis les 2 étapes, puis les 3 étapes, puis les 4 étapes et plus. Au sein de chaque type : d'abord le cycle CFD (MetaTrader 5 en premier, puis les autres plateformes), ensuite le cycle Futures. À prix égal de rang, le plus gros capital est pris en premier.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Comptes À ÉTAPES : il faut d'abord valider l'évaluation, à raison de 10 % par mois. Un objectif de 10 % prend 1 mois, 5 % prend une demi-mois. Un 2 étapes 10 %+5 % met donc 1,5 mois à être financé, et ne rapporte qu'ensuite. La durée exacte est dans l'onglet Détail (colonne Durée d'évaluation) et sa date de financement.</t>
+          <t>Comptes DIRECTS / INSTANT : financés immédiatement, ils rapportent dès la fin du mois d'achat.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ce classeur ne contient QUE les firmes listées sur le site PropFirmMatch.</t>
+          <t>Comptes À ÉTAPES : il faut d'abord valider l'évaluation, à raison de 10 % par mois. Un objectif de 10 % prend 1 mois, 5 % prend une demi-mois. Un 2 étapes 10 %+5 % met donc 1,5 mois à être financé, et ne rapporte qu'ensuite. La durée exacte est dans l'onglet Détail (colonne Durée d'évaluation) et sa date de financement.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Dans ce scénario (10 % / 30 %), la dernière firme est financée vers le 01 mai 2027.</t>
+          <t>Ce classeur ne contient QUE les firmes listées sur le site PropFirmMatch.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Dans ce scénario (10 % / 30 %), la dernière firme est financée vers le 01 avril 2027.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>LES ONGLETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Plan mensuel : date en lettres, firmes achetées, capital financé (déjà validé), capital en cours d'évaluation, payout brut, part firme, salaire net, trésorerie.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Détail des achats : chaque firme, sa date d'achat, son type, sa durée d'évaluation et sa date de financement.</t>
+          <t>Plan mensuel : date en lettres, firmes achetées, capital financé (déjà validé), capital en cours d'évaluation, payout brut, part firme, salaire net, trésorerie.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Détail des achats : chaque firme, sa date d'achat, son type, sa durée d'évaluation et sa date de financement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Paramètres / Graphiques.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Ordre et calendrier calculés pour 10 %/30 %. Colonnes d'argent en formules. Prix hors codes promo. Borne théorique sans échec d'évaluation ni plafond de retrait.</t>
         </is>
@@ -962,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1086,17 +1093,17 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>FundYourFX; The5ers; Thetradercapital</t>
+          <t>Real Trader Fund</t>
         </is>
       </c>
       <c r="C3" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>10000</v>
+        <v>110000</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>323000</v>
+        <v>0</v>
       </c>
       <c r="F3" s="12">
         <f>D3*Paramètres!$B$3</f>
@@ -1111,14 +1118,14 @@
         <v/>
       </c>
       <c r="I3" s="12">
-        <f>I2+H3-686</f>
+        <f>I2+H3-360</f>
         <v/>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1129,17 +1136,17 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>The5ers Crypto; Real Trader Fund</t>
+          <t>XPIPS; Funding Pips; Alpine Funded; FX2 Funding; Ifunds</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>433000</v>
+        <v>1210000</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="F4" s="12">
         <f>D4*Paramètres!$B$3</f>
@@ -1154,14 +1161,14 @@
         <v/>
       </c>
       <c r="I4" s="12">
-        <f>I3+H4-477</f>
+        <f>I3+H4-5522</f>
         <v/>
       </c>
       <c r="J4" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K4" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -1172,17 +1179,17 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>PaidPex; Lux Trading Firm; Finotive Funding; XLTrade; Funded Trader Markets; Sway Funded</t>
+          <t>ADN Broker; FundedHive; FundedForge; BuoyTrade; PaidPex; Lux Trading Firm … (+20)</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>1433000</v>
+        <v>5850000</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>14520000</v>
+        <v>17340000</v>
       </c>
       <c r="F5" s="12">
         <f>D5*Paramètres!$B$3</f>
@@ -1197,14 +1204,14 @@
         <v/>
       </c>
       <c r="I5" s="12">
-        <f>I4+H5-41704</f>
+        <f>I4+H5-121739</f>
         <v/>
       </c>
       <c r="J5" s="9" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K5" s="9" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
@@ -1215,17 +1222,17 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Upcomers; IF Crypto; Instant Funding; Leveraged; Pro Traders Fund; Mainet Funded … (+15)</t>
+          <t>PipFarm; Get Funded Now; Tradeify; BluSky; The Trading Pit Futures; Bulenox … (+47)</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>22853000</v>
+        <v>29590000</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>9095000</v>
+        <v>21038000</v>
       </c>
       <c r="F6" s="12">
         <f>D6*Paramètres!$B$3</f>
@@ -1240,14 +1247,14 @@
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>I5+H6-132467</f>
+        <f>I5+H6-144314</f>
         <v/>
       </c>
       <c r="J6" s="9" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7">
@@ -1256,19 +1263,15 @@
           <t>01 mars 2027</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>FTMO; TradersFlow; The Trading Pit; Ultimate Traders; BrightFunded; Quant Funded … (+47)</t>
-        </is>
-      </c>
+      <c r="B7" s="9" t="inlineStr"/>
       <c r="C7" s="9" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>34288000</v>
+        <v>48208000</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>16340000</v>
+        <v>2420000</v>
       </c>
       <c r="F7" s="12">
         <f>D7*Paramètres!$B$3</f>
@@ -1283,11 +1286,11 @@
         <v/>
       </c>
       <c r="I7" s="12">
-        <f>I6+H7-96601</f>
+        <f>I6+H7-0</f>
         <v/>
       </c>
       <c r="J7" s="9" t="n">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>86</v>
@@ -1304,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>50228000</v>
+        <v>50628000</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>400000</v>
+        <v>0</v>
       </c>
       <c r="F8" s="12">
         <f>D8*Paramètres!$B$3</f>
@@ -1326,48 +1329,9 @@
         <v/>
       </c>
       <c r="J8" s="9" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>01 mai 2027</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr"/>
-      <c r="C9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>50628000</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="12">
-        <f>D9*Paramètres!$B$3</f>
-        <v/>
-      </c>
-      <c r="G9" s="12">
-        <f>F9*Paramètres!$B$4</f>
-        <v/>
-      </c>
-      <c r="H9" s="10">
-        <f>F9-G9</f>
-        <v/>
-      </c>
-      <c r="I9" s="12">
-        <f>I8+H9-0</f>
-        <v/>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>86</v>
-      </c>
-      <c r="K9" s="9" t="n">
         <v>86</v>
       </c>
     </row>
@@ -1462,7 +1426,7 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>FundYourFX</t>
+          <t>Real Trader Fund</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -1477,28 +1441,28 @@
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="n">
-        <v>1</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>01 décembre 2026</t>
+          <t>01 novembre 2026</t>
         </is>
       </c>
       <c r="I2" s="12" t="n">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>514</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>01 novembre 2026</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
@@ -1508,7 +1472,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>The5ers</t>
+          <t>XPIPS</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -1523,28 +1487,28 @@
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
-        </is>
-      </c>
-      <c r="G3" s="15" t="n">
-        <v>1.6</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>19 décembre 2026</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="I3" s="12" t="n">
-        <v>120000</v>
+        <v>400000</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>117</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>01 novembre 2026</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
@@ -1554,12 +1518,12 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Thetradercapital</t>
+          <t>Funding Pips</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -1569,22 +1533,22 @@
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
-        </is>
-      </c>
-      <c r="G4" s="15" t="n">
-        <v>1.5</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>16 décembre 2026</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="I4" s="12" t="n">
-        <v>3000</v>
+        <v>300000</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>55</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="5">
@@ -1600,12 +1564,12 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>The5ers Crypto</t>
+          <t>Alpine Funded</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>cTrader, TradingView</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1615,22 +1579,22 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
-        </is>
-      </c>
-      <c r="G5" s="15" t="n">
-        <v>2</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="I5" s="12" t="n">
-        <v>120000</v>
+        <v>200000</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>117</v>
+        <v>839</v>
       </c>
     </row>
     <row r="6">
@@ -1646,12 +1610,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Real Trader Fund</t>
+          <t>FX2 Funding</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1673,16 +1637,16 @@
         </is>
       </c>
       <c r="I6" s="12" t="n">
-        <v>100000</v>
+        <v>190000</v>
       </c>
       <c r="J6" s="12" t="n">
-        <v>360</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>01 janvier 2027</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1692,12 +1656,12 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>PaidPex</t>
+          <t>Ifunds</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -1707,22 +1671,22 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="n">
-        <v>1</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 décembre 2026</t>
         </is>
       </c>
       <c r="I7" s="12" t="n">
-        <v>6000000</v>
+        <v>10000</v>
       </c>
       <c r="J7" s="12" t="n">
-        <v>11960</v>
+        <v>700</v>
       </c>
     </row>
     <row r="8">
@@ -1738,12 +1702,12 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Lux Trading Firm</t>
+          <t>ADN Broker</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>TradingView</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1753,22 +1717,22 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
-        </is>
-      </c>
-      <c r="G8" s="15" t="n">
-        <v>1</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="I8" s="12" t="n">
-        <v>5000000</v>
+        <v>500000</v>
       </c>
       <c r="J8" s="12" t="n">
-        <v>4995</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="9">
@@ -1784,37 +1748,37 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Finotive Funding</t>
+          <t>FundedHive</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>1.25</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>09 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="I9" s="12" t="n">
-        <v>1400000</v>
+        <v>1000000</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>11200</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10">
@@ -1830,37 +1794,37 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>XLTrade</t>
+          <t>FundedForge</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
-        </is>
-      </c>
-      <c r="G10" s="15" t="n">
-        <v>1</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="I10" s="12" t="n">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>3168</v>
+        <v>650</v>
       </c>
     </row>
     <row r="11">
@@ -1876,37 +1840,37 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Funded Trader Markets</t>
+          <t>BuoyTrade</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker</t>
+          <t xml:space="preserve">MetaTrader </t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
-        </is>
-      </c>
-      <c r="G11" s="15" t="n">
-        <v>0.6</v>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0</v>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>19 janvier 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="I11" s="12" t="n">
-        <v>1000000</v>
+        <v>40000</v>
       </c>
       <c r="J11" s="12" t="n">
-        <v>5436</v>
+        <v>1980</v>
       </c>
     </row>
     <row r="12">
@@ -1922,7 +1886,7 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Sway Funded</t>
+          <t>PaidPex</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -1937,28 +1901,28 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G12" s="15" t="n">
-        <v>1.8</v>
+        <v>1</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>25 février 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I12" s="12" t="n">
-        <v>1000000</v>
+        <v>6000000</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>4945</v>
+        <v>11960</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -1968,12 +1932,12 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Upcomers</t>
+          <t>Lux Trading Firm</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker, DXtr</t>
+          <t>TradingView</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1983,28 +1947,28 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G13" s="15" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>25 février 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I13" s="12" t="n">
-        <v>4000000</v>
+        <v>5000000</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>30795</v>
+        <v>4995</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -2014,12 +1978,12 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>IF Crypto</t>
+          <t>XLTrade</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -2037,20 +2001,20 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I14" s="12" t="n">
         <v>1000000</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>7390</v>
+        <v>3168</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -2060,12 +2024,12 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Instant Funding</t>
+          <t>Funded Trader Markets</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>cTrader, Match-Trader, TradeLocker</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -2079,24 +2043,24 @@
         </is>
       </c>
       <c r="G15" s="15" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>28 février 2027</t>
+          <t>19 janvier 2027</t>
         </is>
       </c>
       <c r="I15" s="12" t="n">
         <v>1000000</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>7390</v>
+        <v>5436</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -2106,12 +2070,12 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Leveraged</t>
+          <t>IF Crypto</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -2121,28 +2085,28 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G16" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I16" s="12" t="n">
         <v>1000000</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>2996</v>
+        <v>7390</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -2152,12 +2116,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Pro Traders Fund</t>
+          <t>Instant Funding</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -2167,28 +2131,28 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G17" s="15" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>07 mars 2027</t>
+          <t>28 janvier 2027</t>
         </is>
       </c>
       <c r="I17" s="12" t="n">
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>4197</v>
+        <v>7390</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B18" s="14" t="inlineStr">
@@ -2198,12 +2162,12 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Mainet Funded</t>
+          <t>Hola Prime</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>cTrader, Match-Trader, TradeLocker</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -2213,28 +2177,28 @@
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G18" s="15" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>10 mars 2027</t>
+          <t>19 janvier 2027</t>
         </is>
       </c>
       <c r="I18" s="12" t="n">
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>2975</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
@@ -2244,12 +2208,12 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Fintokei</t>
+          <t>E8 Perpetuals</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradingView</t>
+          <t>MetaTrader 5, cTrader, TradeLocker</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -2259,28 +2223,28 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G19" s="15" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>04 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I19" s="12" t="n">
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="J19" s="12" t="n">
-        <v>2933</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
@@ -2290,12 +2254,12 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>ADN Broker</t>
+          <t>E8 Markets</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -2305,28 +2269,28 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="n">
-        <v>0</v>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>0.6</v>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>19 janvier 2027</t>
         </is>
       </c>
       <c r="I20" s="12" t="n">
         <v>500000</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>50000</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
@@ -2336,12 +2300,12 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Hola Prime</t>
+          <t>Foxx Funded</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, TradeLocker</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
@@ -2355,24 +2319,24 @@
         </is>
       </c>
       <c r="G21" s="15" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>19 février 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I21" s="12" t="n">
         <v>500000</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>1236</v>
+        <v>1990</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
@@ -2382,12 +2346,12 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>E8 Perpetuals</t>
+          <t>Quantum Funding</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradeLocker</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
@@ -2405,20 +2369,20 @@
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I22" s="12" t="n">
         <v>500000</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>1300</v>
+        <v>2145</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
@@ -2428,12 +2392,12 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>E8 Markets</t>
+          <t>Blue Guardian</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
+          <t>MetaTrader 5, Match-Trader, TradeLocker,</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
@@ -2447,24 +2411,24 @@
         </is>
       </c>
       <c r="G23" s="15" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>19 février 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I23" s="12" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>1300</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
@@ -2474,12 +2438,12 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Foxx Funded</t>
+          <t>FTMO</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>MetaTrader 5, cTrader, TradingView</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -2497,20 +2461,20 @@
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I24" s="12" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>1990</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
@@ -2520,12 +2484,12 @@
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Quantum Funding</t>
+          <t>TradersFlow</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -2543,20 +2507,20 @@
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I25" s="12" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>2145</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
@@ -2566,12 +2530,12 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>IC Funded</t>
+          <t>The Trading Pit</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -2581,28 +2545,28 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G26" s="15" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>16 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I26" s="12" t="n">
-        <v>500000</v>
+        <v>400000</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>2495</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
@@ -2612,12 +2576,12 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Vertex Funding</t>
+          <t>FundYourFX</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -2627,28 +2591,28 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G27" s="15" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>16 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I27" s="12" t="n">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>2525</v>
+        <v>514</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr">
@@ -2658,12 +2622,12 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>FNC Funding</t>
+          <t>FunderPro</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>cTrader, TradeLocker</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2673,28 +2637,28 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G28" s="15" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>13 février 2027</t>
         </is>
       </c>
       <c r="I28" s="12" t="n">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>2625</v>
+        <v>989</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -2704,7 +2668,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Blink Funding</t>
+          <t>Funded Trading Plus</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -2719,28 +2683,28 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G29" s="15" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>16 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I29" s="12" t="n">
-        <v>500000</v>
+        <v>200000</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>1800</v>
+        <v>999</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -2750,12 +2714,12 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>SFX Funded</t>
+          <t>CK Capital</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Match-Trader</t>
+          <t>TradeLocker</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -2765,28 +2729,28 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G30" s="15" t="n">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>10 mars 2027</t>
+          <t>07 février 2027</t>
         </is>
       </c>
       <c r="I30" s="12" t="n">
-        <v>495000</v>
+        <v>200000</v>
       </c>
       <c r="J30" s="12" t="n">
-        <v>2125</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -2796,12 +2760,12 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>XPIPS</t>
+          <t>Ment Funding</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
@@ -2811,11 +2775,11 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>0</v>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>1</v>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
@@ -2823,16 +2787,16 @@
         </is>
       </c>
       <c r="I31" s="12" t="n">
-        <v>400000</v>
+        <v>190000</v>
       </c>
       <c r="J31" s="12" t="n">
-        <v>1596</v>
+        <v>7451</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -2842,12 +2806,12 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Blue Guardian</t>
+          <t>Leveraged Crypto</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader, TradeLocker,</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr">
@@ -2865,20 +2829,20 @@
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I32" s="12" t="n">
-        <v>400000</v>
+        <v>150000</v>
       </c>
       <c r="J32" s="12" t="n">
-        <v>1472</v>
+        <v>980</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>01 février 2027</t>
+          <t>01 janvier 2027</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2888,12 +2852,12 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Atlas Funded</t>
+          <t>Paid To Trade</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, TradeLocker, Rithmic</t>
+          <t>Match-Trader</t>
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr">
@@ -2903,28 +2867,28 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G33" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="I33" s="12" t="n">
-        <v>400000</v>
+        <v>100000</v>
       </c>
       <c r="J33" s="12" t="n">
-        <v>1182</v>
+        <v>699</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2934,17 +2898,17 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>FTMO</t>
+          <t>PipFarm</t>
         </is>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradingView</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr">
@@ -2953,24 +2917,24 @@
         </is>
       </c>
       <c r="G34" s="15" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>07 mars 2027</t>
         </is>
       </c>
       <c r="I34" s="12" t="n">
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="J34" s="12" t="n">
-        <v>1996</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -2980,17 +2944,17 @@
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>TradersFlow</t>
+          <t>Get Funded Now</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t xml:space="preserve">Not named on the official site </t>
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
@@ -3003,40 +2967,40 @@
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>01 mars 2027</t>
         </is>
       </c>
       <c r="I35" s="12" t="n">
         <v>400000</v>
       </c>
       <c r="J35" s="12" t="n">
-        <v>2018</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>CFD</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Futures</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>The Trading Pit</t>
+          <t>Tradeify</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>MT5</t>
+          <t>NinjaTrader, Tradovate, Quantower, Tradi</t>
         </is>
       </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
@@ -3045,162 +3009,162 @@
         </is>
       </c>
       <c r="G36" s="15" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>19 février 2027</t>
         </is>
       </c>
       <c r="I36" s="12" t="n">
-        <v>400000</v>
+        <v>1650000</v>
       </c>
       <c r="J36" s="12" t="n">
-        <v>2276</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>Futures</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>BluSky</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>NinjaTrader, Tradovate, Rithmic, Quantow</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
+        <is>
           <t>01 mars 2027</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>CFD</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Ultimate Traders</t>
-        </is>
-      </c>
-      <c r="D37" s="9" t="inlineStr">
-        <is>
-          <t>MT5</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>2 étapes</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
-        <is>
-          <t>16 avril 2027</t>
-        </is>
-      </c>
       <c r="I37" s="12" t="n">
-        <v>400000</v>
+        <v>900000</v>
       </c>
       <c r="J37" s="12" t="n">
-        <v>1798</v>
+        <v>672</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>Futures</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>The Trading Pit Futures</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>NinjaTrader, Tradovate, Rithmic, Quantow</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>1 étape</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
           <t>01 mars 2027</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>CFD</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>BrightFunded</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>cTrader, DXtrade</t>
-        </is>
-      </c>
-      <c r="E38" s="9" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>2 étapes</t>
-        </is>
-      </c>
-      <c r="G38" s="15" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
-        <is>
-          <t>10 avril 2027</t>
-        </is>
-      </c>
       <c r="I38" s="12" t="n">
-        <v>400000</v>
+        <v>750000</v>
       </c>
       <c r="J38" s="12" t="n">
-        <v>1894</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>CFD</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>Futures</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>Quant Funded</t>
+          <t>Bulenox</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>NinjaTrader, Rithmic, Quantower</t>
         </is>
       </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>1 étape</t>
         </is>
       </c>
       <c r="G39" s="15" t="n">
-        <v>1.5</v>
+        <v>0.6</v>
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>19 février 2027</t>
         </is>
       </c>
       <c r="I39" s="12" t="n">
-        <v>400000</v>
+        <v>750000</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>1996</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -3210,12 +3174,12 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Audacity Capital</t>
+          <t>Upcomers</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, DXtrade</t>
+          <t>cTrader, Match-Trader, TradeLocker, DXtr</t>
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr">
@@ -3229,24 +3193,24 @@
         </is>
       </c>
       <c r="G40" s="15" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>25 février 2027</t>
         </is>
       </c>
       <c r="I40" s="12" t="n">
-        <v>400000</v>
+        <v>4000000</v>
       </c>
       <c r="J40" s="12" t="n">
-        <v>2098</v>
+        <v>30795</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3256,12 +3220,12 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>WSFunded</t>
+          <t>Finotive Funding</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>MetaTrader 5, Match-Trader</t>
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr">
@@ -3275,24 +3239,24 @@
         </is>
       </c>
       <c r="G41" s="15" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>09 mars 2027</t>
         </is>
       </c>
       <c r="I41" s="12" t="n">
-        <v>400000</v>
+        <v>1400000</v>
       </c>
       <c r="J41" s="12" t="n">
-        <v>2236</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -3302,12 +3266,12 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>AquaFunded</t>
+          <t>Sway Funded</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, TradeLocker, Rith</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E42" s="9" t="inlineStr">
@@ -3317,28 +3281,28 @@
       </c>
       <c r="F42" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G42" s="15" t="n">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>19 avril 2027</t>
+          <t>25 mars 2027</t>
         </is>
       </c>
       <c r="I42" s="12" t="n">
-        <v>400000</v>
+        <v>1000000</v>
       </c>
       <c r="J42" s="12" t="n">
-        <v>1354</v>
+        <v>4945</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
@@ -3348,12 +3312,12 @@
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Orion Funded</t>
+          <t>Pro Traders Fund</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E43" s="9" t="inlineStr">
@@ -3363,28 +3327,28 @@
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G43" s="15" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>01 mai 2027</t>
+          <t>07 mars 2027</t>
         </is>
       </c>
       <c r="I43" s="12" t="n">
-        <v>400000</v>
+        <v>900000</v>
       </c>
       <c r="J43" s="12" t="n">
-        <v>1478</v>
+        <v>4197</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -3394,12 +3358,12 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Get Crypto Funded</t>
+          <t>Mainet Funded</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -3409,28 +3373,28 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G44" s="15" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>25 avril 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I44" s="12" t="n">
-        <v>400000</v>
+        <v>700000</v>
       </c>
       <c r="J44" s="12" t="n">
-        <v>1648</v>
+        <v>2975</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
@@ -3440,12 +3404,12 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Funding Pips</t>
+          <t>IC Funded</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
@@ -3455,28 +3419,28 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G45" s="9" t="n">
-        <v>0</v>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>1.5</v>
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I45" s="12" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="J45" s="12" t="n">
-        <v>1332</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -3486,12 +3450,12 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Clarity Traders</t>
+          <t>Vertex Funding</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, TradeLocker</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
@@ -3505,24 +3469,24 @@
         </is>
       </c>
       <c r="G46" s="15" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>10 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I46" s="12" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="J46" s="12" t="n">
-        <v>1399</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -3532,12 +3496,12 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Prop Number One</t>
+          <t>FNC Funding</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -3551,24 +3515,24 @@
         </is>
       </c>
       <c r="G47" s="15" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>01 avril 2027</t>
         </is>
       </c>
       <c r="I47" s="12" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="J47" s="12" t="n">
-        <v>1592</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -3578,12 +3542,12 @@
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Tradeify 247</t>
+          <t>SFX Funded</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, DXtrade</t>
+          <t>Match-Trader</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
@@ -3597,24 +3561,24 @@
         </is>
       </c>
       <c r="G48" s="15" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I48" s="12" t="n">
-        <v>300000</v>
+        <v>495000</v>
       </c>
       <c r="J48" s="12" t="n">
-        <v>1740</v>
+        <v>2125</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
@@ -3624,12 +3588,12 @@
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>Myfundedcapital</t>
+          <t>Ultimate Traders</t>
         </is>
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E49" s="9" t="inlineStr">
@@ -3647,20 +3611,20 @@
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I49" s="12" t="n">
-        <v>300000</v>
+        <v>400000</v>
       </c>
       <c r="J49" s="12" t="n">
-        <v>1905</v>
+        <v>1798</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
@@ -3670,12 +3634,12 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>Alpine Funded</t>
+          <t>BrightFunded</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, cTrader</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
@@ -3685,28 +3649,28 @@
       </c>
       <c r="F50" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G50" s="9" t="n">
-        <v>0</v>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="n">
+        <v>1.3</v>
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I50" s="12" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="J50" s="12" t="n">
-        <v>839</v>
+        <v>1894</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
@@ -3716,12 +3680,12 @@
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>FunderPro</t>
+          <t>Quant Funded</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>cTrader, TradeLocker</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -3731,28 +3695,28 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G51" s="15" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="H51" s="9" t="inlineStr">
         <is>
-          <t>13 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I51" s="12" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="J51" s="12" t="n">
-        <v>989</v>
+        <v>1996</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -3762,12 +3726,12 @@
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Funded Trading Plus</t>
+          <t>Audacity Capital</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>MetaTrader 5, DXtrade</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
@@ -3777,28 +3741,28 @@
       </c>
       <c r="F52" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G52" s="15" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I52" s="12" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="J52" s="12" t="n">
-        <v>999</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -3808,12 +3772,12 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>CK Capital</t>
+          <t>WSFunded</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>TradeLocker</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -3823,28 +3787,28 @@
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G53" s="15" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>07 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I53" s="12" t="n">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="J53" s="12" t="n">
-        <v>1056</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
@@ -3854,12 +3818,12 @@
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>NowTradeFunded</t>
+          <t>Clarity Traders</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>MetaTrader 5, TradeLocker</t>
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr">
@@ -3873,24 +3837,24 @@
         </is>
       </c>
       <c r="G54" s="15" t="n">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
-          <t>22 avril 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I54" s="12" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="J54" s="12" t="n">
-        <v>900</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B55" s="14" t="inlineStr">
@@ -3900,12 +3864,12 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Crypto Fund Trader</t>
+          <t>Prop Number One</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5, Match-Trader</t>
+          <t>MetaTrader 5, cTrader, Match-Trader, Tra</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
@@ -3919,24 +3883,24 @@
         </is>
       </c>
       <c r="G55" s="15" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="H55" s="9" t="inlineStr">
         <is>
-          <t>10 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I55" s="12" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="J55" s="12" t="n">
-        <v>1250</v>
+        <v>1592</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
@@ -3946,12 +3910,12 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>FX2 Funding</t>
+          <t>Tradeify 247</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>cTrader, DXtrade</t>
+          <t>MetaTrader 5, DXtrade</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
@@ -3961,28 +3925,28 @@
       </c>
       <c r="F56" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G56" s="9" t="n">
-        <v>0</v>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="n">
+        <v>1.5</v>
       </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I56" s="12" t="n">
-        <v>190000</v>
+        <v>300000</v>
       </c>
       <c r="J56" s="12" t="n">
-        <v>1055</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
@@ -3992,12 +3956,12 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Ment Funding</t>
+          <t>Myfundedcapital</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>cTrader, DXtrade</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -4007,28 +3971,28 @@
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G57" s="15" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I57" s="12" t="n">
-        <v>190000</v>
+        <v>300000</v>
       </c>
       <c r="J57" s="12" t="n">
-        <v>7451</v>
+        <v>1905</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
@@ -4038,12 +4002,12 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Leveraged Crypto</t>
+          <t>NowTradeFunded</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>cTrader</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
@@ -4053,28 +4017,28 @@
       </c>
       <c r="F58" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G58" s="15" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>22 mars 2027</t>
         </is>
       </c>
       <c r="I58" s="12" t="n">
-        <v>150000</v>
+        <v>200000</v>
       </c>
       <c r="J58" s="12" t="n">
-        <v>980</v>
+        <v>900</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B59" s="14" t="inlineStr">
@@ -4084,12 +4048,12 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Paid To Trade</t>
+          <t>Crypto Fund Trader</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Match-Trader</t>
+          <t>MetaTrader 5, Match-Trader</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
@@ -4099,28 +4063,28 @@
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G59" s="15" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I59" s="12" t="n">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="J59" s="12" t="n">
-        <v>699</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B60" s="14" t="inlineStr">
@@ -4153,7 +4117,7 @@
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I60" s="12" t="n">
@@ -4166,7 +4130,7 @@
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B61" s="14" t="inlineStr">
@@ -4199,7 +4163,7 @@
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I61" s="12" t="n">
@@ -4212,7 +4176,7 @@
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B62" s="14" t="inlineStr">
@@ -4245,7 +4209,7 @@
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I62" s="12" t="n">
@@ -4258,7 +4222,7 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
@@ -4291,7 +4255,7 @@
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I63" s="12" t="n">
@@ -4304,7 +4268,7 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
@@ -4314,12 +4278,12 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Ifunds</t>
+          <t>Thetradercapital</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>MetaTrader 5</t>
+          <t>MT5</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
@@ -4329,28 +4293,28 @@
       </c>
       <c r="F64" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G64" s="9" t="n">
-        <v>0</v>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="n">
+        <v>1.5</v>
       </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I64" s="12" t="n">
-        <v>10000</v>
+        <v>3000</v>
       </c>
       <c r="J64" s="12" t="n">
-        <v>700</v>
+        <v>55</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
@@ -4360,12 +4324,12 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>FundedHive</t>
+          <t>Tradexprop</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>cTrader, DXtrade</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -4375,28 +4339,28 @@
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="n">
-        <v>0</v>
+          <t>2 étapes</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="n">
+        <v>1.5</v>
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I65" s="12" t="n">
         <v>1000000</v>
       </c>
       <c r="J65" s="12" t="n">
-        <v>349</v>
+        <v>6150</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
@@ -4406,12 +4370,12 @@
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>Tradexprop</t>
+          <t>GoFunding</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>cTrader, DXtrade</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
@@ -4429,20 +4393,20 @@
       </c>
       <c r="H66" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I66" s="12" t="n">
-        <v>1000000</v>
+        <v>800000</v>
       </c>
       <c r="J66" s="12" t="n">
-        <v>6150</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
@@ -4452,7 +4416,7 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>GoFunding</t>
+          <t>Nordic Funder</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -4475,20 +4439,20 @@
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I67" s="12" t="n">
-        <v>800000</v>
+        <v>500000</v>
       </c>
       <c r="J67" s="12" t="n">
-        <v>3600</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
@@ -4498,12 +4462,12 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>PipFarm</t>
+          <t>Mockapital</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>cTrader</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
@@ -4513,28 +4477,28 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G68" s="15" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
-          <t>07 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I68" s="12" t="n">
-        <v>600000</v>
+        <v>300000</v>
       </c>
       <c r="J68" s="12" t="n">
-        <v>2360</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
@@ -4544,12 +4508,12 @@
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Nordic Funder</t>
+          <t>The Concept Trading</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>TradeLocker</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
@@ -4567,20 +4531,20 @@
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I69" s="12" t="n">
-        <v>500000</v>
+        <v>300000</v>
       </c>
       <c r="J69" s="12" t="n">
-        <v>2450</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
@@ -4590,12 +4554,12 @@
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>Get Funded Now</t>
+          <t>FundingRock</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not named on the official site </t>
+          <t>cTrader, TradeLocker</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
@@ -4605,28 +4569,28 @@
       </c>
       <c r="F70" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G70" s="15" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>04 mars 2027</t>
         </is>
       </c>
       <c r="I70" s="12" t="n">
-        <v>400000</v>
+        <v>200000</v>
       </c>
       <c r="J70" s="12" t="n">
-        <v>2625</v>
+        <v>700</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
@@ -4636,12 +4600,12 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>Lark Funding</t>
+          <t>TradersEdgeFX</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t xml:space="preserve">Not named anywhere on the public site </t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
@@ -4651,28 +4615,28 @@
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>3 étapes</t>
+          <t>2 étapes</t>
         </is>
       </c>
       <c r="G71" s="15" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>07 avril 2027</t>
+          <t>10 mars 2027</t>
         </is>
       </c>
       <c r="I71" s="12" t="n">
-        <v>400000</v>
+        <v>200000</v>
       </c>
       <c r="J71" s="12" t="n">
-        <v>1400</v>
+        <v>899</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B72" s="14" t="inlineStr">
@@ -4682,12 +4646,12 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Mockapital</t>
+          <t>Super Funded</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>cTrader, Match-Trader, DXtrade</t>
+          <t>TradeLocker, DXtrade</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
@@ -4705,20 +4669,20 @@
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I72" s="12" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="J72" s="12" t="n">
-        <v>1450</v>
+        <v>999</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B73" s="14" t="inlineStr">
@@ -4728,12 +4692,12 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>The Concept Trading</t>
+          <t>FT9JA</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>TradeLocker</t>
+          <t xml:space="preserve">Broker accounts at IC Markets and FXTM </t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
@@ -4751,20 +4715,20 @@
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I73" s="12" t="n">
-        <v>300000</v>
+        <v>25000</v>
       </c>
       <c r="J73" s="12" t="n">
-        <v>15000</v>
+        <v>141</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
@@ -4774,12 +4738,12 @@
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>FundingRock</t>
+          <t>LevaFX</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>cTrader, TradeLocker</t>
+          <t xml:space="preserve">Proprietary 'LEVA Terminal' </t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
@@ -4793,39 +4757,39 @@
         </is>
       </c>
       <c r="G74" s="15" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="H74" s="9" t="inlineStr">
         <is>
-          <t>04 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I74" s="12" t="n">
-        <v>200000</v>
+        <v>25000</v>
       </c>
       <c r="J74" s="12" t="n">
-        <v>700</v>
+        <v>149</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B75" s="14" t="inlineStr">
-        <is>
-          <t>CFD</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>Futures</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>TradersEdgeFX</t>
+          <t>HyroTrader</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not named anywhere on the public site </t>
+          <t xml:space="preserve">Bybit demo </t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
@@ -4839,24 +4803,24 @@
         </is>
       </c>
       <c r="G75" s="15" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>10 avril 2027</t>
+          <t>25 mars 2027</t>
         </is>
       </c>
       <c r="I75" s="12" t="n">
         <v>200000</v>
       </c>
       <c r="J75" s="12" t="n">
-        <v>899</v>
+        <v>999</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B76" s="14" t="inlineStr">
@@ -4866,43 +4830,43 @@
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Super Funded</t>
+          <t>Leveraged</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>TradeLocker, DXtrade</t>
+          <t>MetaTrader 5, cTrader</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G76" s="15" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>01 avril 2027</t>
         </is>
       </c>
       <c r="I76" s="12" t="n">
-        <v>200000</v>
+        <v>1000000</v>
       </c>
       <c r="J76" s="12" t="n">
-        <v>999</v>
+        <v>2996</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B77" s="14" t="inlineStr">
@@ -4912,17 +4876,17 @@
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>Turbo Trade Fund</t>
+          <t>Fintokei</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Match-Trader</t>
+          <t>MetaTrader 5, cTrader, TradingView</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr">
@@ -4931,24 +4895,24 @@
         </is>
       </c>
       <c r="G77" s="15" t="n">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>04 mars 2027</t>
         </is>
       </c>
       <c r="I77" s="12" t="n">
-        <v>200000</v>
+        <v>700000</v>
       </c>
       <c r="J77" s="12" t="n">
-        <v>799</v>
+        <v>2933</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
@@ -4958,7 +4922,7 @@
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>FundedForge</t>
+          <t>Blink Funding</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -4968,33 +4932,33 @@
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G78" s="9" t="n">
-        <v>0</v>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G78" s="15" t="n">
+        <v>1.5</v>
       </c>
       <c r="H78" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I78" s="12" t="n">
-        <v>100000</v>
+        <v>500000</v>
       </c>
       <c r="J78" s="12" t="n">
-        <v>650</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B79" s="14" t="inlineStr">
@@ -5004,43 +4968,43 @@
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>BuoyTrade</t>
+          <t>Atlas Funded</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MetaTrader </t>
+          <t>MetaTrader 5, TradeLocker, Rithmic</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="G79" s="9" t="n">
-        <v>0</v>
+          <t>3 étapes</t>
+        </is>
+      </c>
+      <c r="G79" s="15" t="n">
+        <v>2</v>
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 avril 2027</t>
         </is>
       </c>
       <c r="I79" s="12" t="n">
-        <v>40000</v>
+        <v>400000</v>
       </c>
       <c r="J79" s="12" t="n">
-        <v>1980</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B80" s="14" t="inlineStr">
@@ -5050,43 +5014,43 @@
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>FT9JA</t>
+          <t>AquaFunded</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Broker accounts at IC Markets and FXTM </t>
+          <t>MetaTrader 5, cTrader, TradeLocker, Rith</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G80" s="15" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="H80" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>19 mars 2027</t>
         </is>
       </c>
       <c r="I80" s="12" t="n">
-        <v>25000</v>
+        <v>400000</v>
       </c>
       <c r="J80" s="12" t="n">
-        <v>141</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
+          <t>01 février 2027</t>
         </is>
       </c>
       <c r="B81" s="14" t="inlineStr">
@@ -5096,164 +5060,164 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>LevaFX</t>
+          <t>Orion Funded</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Proprietary 'LEVA Terminal' </t>
+          <t>cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G81" s="15" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H81" s="9" t="inlineStr">
         <is>
-          <t>16 avril 2027</t>
+          <t>01 avril 2027</t>
         </is>
       </c>
       <c r="I81" s="12" t="n">
-        <v>25000</v>
+        <v>400000</v>
       </c>
       <c r="J81" s="12" t="n">
-        <v>149</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B82" s="16" t="inlineStr">
-        <is>
-          <t>Futures</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B82" s="14" t="inlineStr">
+        <is>
+          <t>CFD</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>Tradeify</t>
+          <t>Get Crypto Funded</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>NinjaTrader, Tradovate, Quantower, Tradi</t>
+          <t>MetaTrader 5, cTrader, Match-Trader</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G82" s="15" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="H82" s="9" t="inlineStr">
         <is>
-          <t>19 mars 2027</t>
+          <t>25 mars 2027</t>
         </is>
       </c>
       <c r="I82" s="12" t="n">
-        <v>1650000</v>
+        <v>400000</v>
       </c>
       <c r="J82" s="12" t="n">
-        <v>2114</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B83" s="16" t="inlineStr">
-        <is>
-          <t>Futures</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B83" s="14" t="inlineStr">
+        <is>
+          <t>CFD</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>BluSky</t>
+          <t>The5ers</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>NinjaTrader, Tradovate, Rithmic, Quantow</t>
+          <t>MetaTrader 5</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G83" s="15" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>01 avril 2027</t>
+          <t>19 mars 2027</t>
         </is>
       </c>
       <c r="I83" s="12" t="n">
-        <v>900000</v>
+        <v>120000</v>
       </c>
       <c r="J83" s="12" t="n">
-        <v>672</v>
+        <v>117</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B84" s="16" t="inlineStr">
-        <is>
-          <t>Futures</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B84" s="14" t="inlineStr">
+        <is>
+          <t>CFD</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>The Trading Pit Futures</t>
+          <t>The5ers Crypto</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>NinjaTrader, Tradovate, Rithmic, Quantow</t>
+          <t>cTrader, TradingView</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G84" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H84" s="9" t="inlineStr">
         <is>
@@ -5261,31 +5225,31 @@
         </is>
       </c>
       <c r="I84" s="12" t="n">
-        <v>750000</v>
+        <v>120000</v>
       </c>
       <c r="J84" s="12" t="n">
-        <v>1445</v>
+        <v>117</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B85" s="16" t="inlineStr">
-        <is>
-          <t>Futures</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>CFD</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>Bulenox</t>
+          <t>Lark Funding</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>NinjaTrader, Rithmic, Quantower</t>
+          <t>cTrader, Match-Trader, DXtrade</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -5295,43 +5259,43 @@
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>1 étape</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G85" s="15" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="H85" s="9" t="inlineStr">
         <is>
-          <t>19 mars 2027</t>
+          <t>07 mars 2027</t>
         </is>
       </c>
       <c r="I85" s="12" t="n">
-        <v>750000</v>
+        <v>400000</v>
       </c>
       <c r="J85" s="12" t="n">
-        <v>1625</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>01 mars 2027</t>
-        </is>
-      </c>
-      <c r="B86" s="16" t="inlineStr">
-        <is>
-          <t>Futures</t>
+          <t>01 février 2027</t>
+        </is>
+      </c>
+      <c r="B86" s="14" t="inlineStr">
+        <is>
+          <t>CFD</t>
         </is>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>HyroTrader</t>
+          <t>Turbo Trade Fund</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bybit demo </t>
+          <t>Match-Trader</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
@@ -5341,22 +5305,22 @@
       </c>
       <c r="F86" s="9" t="inlineStr">
         <is>
-          <t>2 étapes</t>
+          <t>3 étapes</t>
         </is>
       </c>
       <c r="G86" s="15" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="H86" s="9" t="inlineStr">
         <is>
-          <t>25 avril 2027</t>
+          <t>16 mars 2027</t>
         </is>
       </c>
       <c r="I86" s="12" t="n">
         <v>200000</v>
       </c>
       <c r="J86" s="12" t="n">
-        <v>999</v>
+        <v>799</v>
       </c>
     </row>
   </sheetData>

</xml_diff>